<commit_message>
Implement expense audit agent with receipt validation and policy tools; add tests for error handling
</commit_message>
<xml_diff>
--- a/Defect_Tracker Template_v0.1 (1).xlsx
+++ b/Defect_Tracker Template_v0.1 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI-Agent-Coordination-Engine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C2B141-DB86-48FC-995F-76BFF104637B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748C43A4-FA13-46B0-BA77-7855F232A15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
   <si>
     <t>Sl No</t>
   </si>
@@ -87,6 +87,30 @@
   </si>
   <si>
     <t>Closed</t>
+  </si>
+  <si>
+    <t>The Receipt Validation Tool was invoked twice during a single expense audit because it was both directly executed and registered as a Gemini-callable tool.</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>19-09-20226</t>
+  </si>
+  <si>
+    <t>The subsequent CLI test showed one direct receipt validation and successful policy retrieval. The duplicate invocation was resolved in the observed run.</t>
+  </si>
+  <si>
+    <t>During an expense audit with a zero receipt amount, the Receipt Validation Tool correctly flagged the invalid amount, but the AI audit did not complete.</t>
+  </si>
+  <si>
+    <t>Receipt validation output was confirmed. Further investigation of the AI service failure is pending a rerun and exception diagnosis.</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Removed validate_receipt from the Gemini registered tools list while retaining direct execution for receipt validation.</t>
   </si>
 </sst>
 </file>
@@ -194,9 +218,6 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -215,7 +236,10 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -528,321 +552,364 @@
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultColWidth="17.54296875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.1796875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="42.1796875" style="4" customWidth="1"/>
-    <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="21.81640625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="16.81640625" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="17.54296875" style="4"/>
+    <col min="1" max="1" width="6.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="42.1796875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="16" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="24.90625" style="3" customWidth="1"/>
+    <col min="9" max="10" width="21.81640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="23" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="17.54296875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="31" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="31" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="100" x14ac:dyDescent="0.3">
-      <c r="A2" s="8">
+    <row r="2" spans="1:11" ht="113.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>46267</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="7" t="s">
         <v>9</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="8">
         <v>46267</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="7" t="s">
         <v>21</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+    <row r="3" spans="1:11" ht="129" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="8">
+        <v>46284</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="104.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="8">
+        <v>46284</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="8">
+        <v>46284</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="7"/>
     </row>
     <row r="5" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="6"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="6"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="5"/>
     </row>
     <row r="10" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="6"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="5"/>
     </row>
     <row r="11" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="6"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="6"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="6"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="5"/>
     </row>
     <row r="17" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="6"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="5"/>
     </row>
     <row r="18" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="6"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="5"/>
     </row>
     <row r="19" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="6"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -890,7 +957,7 @@
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
     </row>
@@ -901,6 +968,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1032,12 +1105,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1048,6 +1115,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1065,15 +1141,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat: Implement expense submission form and integrate AI audit agent
- Added a new HTML template for submitting expense claims with validation and preview features.
- Created unit tests for refined classification and policy reasoning in the expense audit agent.
- Developed the main Flask application to handle expense submissions, including validation and AI integration.
- Established health check API for application status monitoring.
</commit_message>
<xml_diff>
--- a/Defect_Tracker Template_v0.1 (1).xlsx
+++ b/Defect_Tracker Template_v0.1 (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI-Agent-Coordination-Engine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{748C43A4-FA13-46B0-BA77-7855F232A15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE970701-1AB7-424C-8230-1A7133E3E56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
   <si>
     <t>Sl No</t>
   </si>
@@ -104,13 +104,16 @@
     <t>During an expense audit with a zero receipt amount, the Receipt Validation Tool correctly flagged the invalid amount, but the AI audit did not complete.</t>
   </si>
   <si>
-    <t>Receipt validation output was confirmed. Further investigation of the AI service failure is pending a rerun and exception diagnosis.</t>
-  </si>
-  <si>
     <t>Open</t>
   </si>
   <si>
-    <t>Removed validate_receipt from the Gemini registered tools list while retaining direct execution for receipt validation.</t>
+    <t>Removed validate_receipt from the Gemini registered tools list while retaining direct execution of receipt validation in the expense audit workflow.</t>
+  </si>
+  <si>
+    <t>Confirmed that the Receipt Validation Tool correctly detected the invalid amount. Further investigation into the subsequent AI service failure is pending, along with a successful end-to-end rerun.</t>
+  </si>
+  <si>
+    <t>Receipt validation behavior was confirmed, but the complete AI audit remains unverified due to a subsequent service/API failure. Retesting is required after investigating the failure.</t>
   </si>
 </sst>
 </file>
@@ -658,7 +661,7 @@
         <v>9</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>24</v>
@@ -670,7 +673,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="104.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="197" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -693,15 +696,17 @@
         <v>9</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I4" s="8">
         <v>46284</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="K4" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
@@ -968,12 +973,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1105,6 +1104,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1115,15 +1120,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1141,6 +1137,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
chore: Update .gitignore and remove obsolete files; add new agent architecture documentation
</commit_message>
<xml_diff>
--- a/Defect_Tracker Template_v0.1 (1).xlsx
+++ b/Defect_Tracker Template_v0.1 (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI-Agent-Coordination-Engine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE970701-1AB7-424C-8230-1A7133E3E56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1DAE9BA-A508-4793-BB0E-7FC870BC9447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="41">
   <si>
     <t>Sl No</t>
   </si>
@@ -114,13 +114,46 @@
   </si>
   <si>
     <t>Receipt validation behavior was confirmed, but the complete AI audit remains unverified due to a subsequent service/API failure. Retesting is required after investigating the failure.</t>
+  </si>
+  <si>
+    <t>Specialized agent failure in Coordinator workflow (e.g. PolicyAgent exception) previously caused downstream workflow failure instead of isolated error handling and transparent error reporting.</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Added try-except blocks around each specialized agent invocation in CoordinatorAgent.run_audit(). Recorded individual agent status ('Failed' vs 'Completed') and formatted user-friendly error strings passed downstream without crashing the pipeline.</t>
+  </si>
+  <si>
+    <t>Verified via automated unit test test_agent_failure in tests/test_m3_workflow.py. Policy status set to 'Failed', remaining workflow completed gracefully.</t>
+  </si>
+  <si>
+    <t>Follow-up chat queries using CoordinatorAgent.handle_follow_up() failed with unhandled exception when invoked with an invalid or expired session_id.</t>
+  </si>
+  <si>
+    <t>Added explicit check in handle_follow_up() to query SESSION_STORE.get(session_id). If missing, immediately returns 'No active session context found. Please submit an expense first.' before invoking LLM.</t>
+  </si>
+  <si>
+    <t>Verified via automated unit test test_missing_context in tests/test_m3_workflow.py. Returned exact user-friendly message instantly.</t>
+  </si>
+  <si>
+    <t>Gemini API 429 RESOURCE_EXHAUSTED rate-limit errors during follow-up chat conversations exposed technical error messages and raw status codes to the user interface.</t>
+  </si>
+  <si>
+    <t>Added handling in CoordinatorAgent.handle_follow_up() to catch 429/quota exceptions via get_user_friendly_error(), return the user-friendly fallback message 'The AI service has temporarily reached its usage limit. Please try again later.', and preserve the existing SESSION_STORE context. Scope: handle_follow_up() path only. Error handling in run_audit() and the web application layer has not been separately re-tested against live 429 responses in Milestone 3.</t>
+  </si>
+  <si>
+    <t>Fix verified by mocked automated unit test test_gemini_429_quota_exhaustion_in_chat in tests/test_m3_workflow.py. Verified behaviours: 429 exception intercepted, raw error message suppressed, session data preserved. Coverage is limited to the handle_follow_up() code path and mocked exception; live API quota exhaustion and other routes remain unverified.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -177,6 +210,10 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -219,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -243,6 +280,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -562,7 +605,7 @@
     <col min="5" max="5" width="16" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.54296875" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.453125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="24.90625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="31.81640625" style="3" customWidth="1"/>
     <col min="9" max="10" width="21.81640625" style="3" customWidth="1"/>
     <col min="11" max="11" width="23" style="3" customWidth="1"/>
     <col min="12" max="16384" width="17.54296875" style="3"/>
@@ -708,44 +751,110 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="5"/>
+    <row r="5" spans="1:11" ht="198.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="11">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="12">
+        <v>46293</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" s="12">
+        <v>46294</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="192" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="11">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="12">
+        <v>46294</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="12">
+        <v>46295</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="325.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="11">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="12">
+        <v>46296</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="12">
+        <v>46297</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="15.5" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
@@ -973,6 +1082,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1104,12 +1219,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1120,6 +1229,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1137,15 +1255,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>

</xml_diff>